<commit_message>
Korp Filial 05/2026: fechamento patrimonial revisado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017VLoTgLZUjFbc7Wvyz5oBv
</commit_message>
<xml_diff>
--- a/Korp/Filial/2026-05/Fechamento_Folha_Korp_Filial_05-2026.xlsx
+++ b/Korp/Filial/2026-05/Fechamento_Folha_Korp_Filial_05-2026.xlsx
@@ -708,7 +708,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Liquido do extrato 05/2026: 83.431,14 (sem rescisões). Situação: TXT corrigido gerado e importado na Korp.</t>
+          <t>Folha 05/2026. Líquido do extrato: 83.431,14 (sem rescisões). TXT corrigido importado na Korp. Sem lançamentos de competência de outros meses.</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>78487.18000000001</v>
+        <v>78487.17999999999</v>
       </c>
       <c r="D5" s="10" t="n">
         <v>78065.32000000001</v>
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>-188.7600000000002</v>
+        <v>-188.76</v>
       </c>
       <c r="D7" s="10" t="n">
         <v>4146.44</v>

</xml_diff>

<commit_message>
Planilhas Korp: gravar valores calculados em vez de fórmulas (visualizador mostrava vazio)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017VLoTgLZUjFbc7Wvyz5oBv
</commit_message>
<xml_diff>
--- a/Korp/Filial/2026-05/Fechamento_Folha_Korp_Filial_05-2026.xlsx
+++ b/Korp/Filial/2026-05/Fechamento_Folha_Korp_Filial_05-2026.xlsx
@@ -529,9 +529,8 @@
           <t>Salários a Pagar</t>
         </is>
       </c>
-      <c r="C5" s="5">
-        <f>'05-2026'!F5</f>
-        <v/>
+      <c r="C5" s="5" t="n">
+        <v>78487.17999999999</v>
       </c>
     </row>
     <row r="6">
@@ -545,9 +544,8 @@
           <t>Indenizações Trabalhistas (rescisões)</t>
         </is>
       </c>
-      <c r="C6" s="5">
-        <f>'05-2026'!F6</f>
-        <v/>
+      <c r="C6" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -561,9 +559,8 @@
           <t>Férias a Pagar</t>
         </is>
       </c>
-      <c r="C7" s="5">
-        <f>'05-2026'!F7</f>
-        <v/>
+      <c r="C7" s="5" t="n">
+        <v>-188.76</v>
       </c>
     </row>
     <row r="8">
@@ -577,9 +574,8 @@
           <t>Estágios a pagar</t>
         </is>
       </c>
-      <c r="C8" s="5">
-        <f>'05-2026'!F8</f>
-        <v/>
+      <c r="C8" s="5" t="n">
+        <v>5132.72</v>
       </c>
     </row>
     <row r="9">
@@ -593,9 +589,8 @@
           <t>FGTS a Recolher</t>
         </is>
       </c>
-      <c r="C9" s="5">
-        <f>'05-2026'!F9</f>
-        <v/>
+      <c r="C9" s="5" t="n">
+        <v>7558.72</v>
       </c>
     </row>
     <row r="10">
@@ -609,9 +604,8 @@
           <t>INSS a Recolher</t>
         </is>
       </c>
-      <c r="C10" s="5">
-        <f>'05-2026'!F10</f>
-        <v/>
+      <c r="C10" s="5" t="n">
+        <v>34220.29</v>
       </c>
     </row>
     <row r="11">
@@ -625,9 +619,8 @@
           <t>IRRF a Recolher s/ Folha</t>
         </is>
       </c>
-      <c r="C11" s="5">
-        <f>'05-2026'!F11</f>
-        <v/>
+      <c r="C11" s="5" t="n">
+        <v>1039.26</v>
       </c>
     </row>
     <row r="12">
@@ -641,9 +634,8 @@
           <t>Empréstimo a Funcionário (consignado)</t>
         </is>
       </c>
-      <c r="C12" s="5">
-        <f>'05-2026'!F12</f>
-        <v/>
+      <c r="C12" s="5" t="n">
+        <v>1990.95</v>
       </c>
     </row>
     <row r="13">
@@ -657,9 +649,8 @@
           <t>Adiantamento de Férias (ativo)</t>
         </is>
       </c>
-      <c r="C13" s="5">
-        <f>'05-2026'!F13</f>
-        <v/>
+      <c r="C13" s="5" t="n">
+        <v>4926.04</v>
       </c>
     </row>
     <row r="14">
@@ -668,9 +659,10 @@
           <t>Confere com a folha?</t>
         </is>
       </c>
-      <c r="C14" s="7">
-        <f>IF(COUNTIF('05-2026'!H5:H13,"Não")=0,"Sim","Não")</f>
-        <v/>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -779,16 +771,16 @@
       <c r="E5" s="10" t="n">
         <v>421.86</v>
       </c>
-      <c r="F5" s="10">
-        <f>D5+E5</f>
-        <v/>
+      <c r="F5" s="10" t="n">
+        <v>78487.17999999999</v>
       </c>
       <c r="G5" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="8">
-        <f>IF(ABS(C5+G5-F5)&lt;1,"Sim","Não")</f>
-        <v/>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
@@ -816,16 +808,16 @@
       <c r="E6" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="10">
-        <f>D6+E6</f>
-        <v/>
+      <c r="F6" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="G6" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="8">
-        <f>IF(ABS(C6+G6-F6)&lt;1,"Sim","Não")</f>
-        <v/>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
@@ -853,16 +845,16 @@
       <c r="E7" s="10" t="n">
         <v>-4335.2</v>
       </c>
-      <c r="F7" s="10">
-        <f>D7+E7</f>
-        <v/>
+      <c r="F7" s="10" t="n">
+        <v>-188.76</v>
       </c>
       <c r="G7" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="8">
-        <f>IF(ABS(C7+G7-F7)&lt;1,"Sim","Não")</f>
-        <v/>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
@@ -890,16 +882,16 @@
       <c r="E8" s="10" t="n">
         <v>2961.3</v>
       </c>
-      <c r="F8" s="10">
-        <f>D8+E8</f>
-        <v/>
+      <c r="F8" s="10" t="n">
+        <v>5132.72</v>
       </c>
       <c r="G8" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="8">
-        <f>IF(ABS(C8+G8-F8)&lt;1,"Sim","Não")</f>
-        <v/>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
@@ -927,16 +919,16 @@
       <c r="E9" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="10">
-        <f>D9+E9</f>
-        <v/>
+      <c r="F9" s="10" t="n">
+        <v>7558.72</v>
       </c>
       <c r="G9" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="8">
-        <f>IF(ABS(C9+G9-F9)&lt;1,"Sim","Não")</f>
-        <v/>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
       <c r="I9" s="11" t="inlineStr"/>
     </row>
@@ -960,16 +952,16 @@
       <c r="E10" s="10" t="n">
         <v>231.5</v>
       </c>
-      <c r="F10" s="10">
-        <f>D10+E10</f>
-        <v/>
+      <c r="F10" s="10" t="n">
+        <v>34220.29</v>
       </c>
       <c r="G10" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="8">
-        <f>IF(ABS(C10+G10-F10)&lt;1,"Sim","Não")</f>
-        <v/>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
@@ -997,16 +989,16 @@
       <c r="E11" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="10">
-        <f>D11+E11</f>
-        <v/>
+      <c r="F11" s="10" t="n">
+        <v>1039.26</v>
       </c>
       <c r="G11" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="8">
-        <f>IF(ABS(C11+G11-F11)&lt;1,"Sim","Não")</f>
-        <v/>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
       <c r="I11" s="11" t="inlineStr"/>
     </row>
@@ -1030,16 +1022,16 @@
       <c r="E12" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="10">
-        <f>D12+E12</f>
-        <v/>
+      <c r="F12" s="10" t="n">
+        <v>1990.95</v>
       </c>
       <c r="G12" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="8">
-        <f>IF(ABS(C12+G12-F12)&lt;1,"Sim","Não")</f>
-        <v/>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
       <c r="I12" s="11" t="inlineStr"/>
     </row>
@@ -1063,16 +1055,16 @@
       <c r="E13" s="10" t="n">
         <v>4926.04</v>
       </c>
-      <c r="F13" s="10">
-        <f>D13+E13</f>
-        <v/>
+      <c r="F13" s="10" t="n">
+        <v>4926.04</v>
       </c>
       <c r="G13" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="8">
-        <f>IF(ABS(C13+G13-F13)&lt;1,"Sim","Não")</f>
-        <v/>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
@@ -1093,21 +1085,17 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="C16" s="12">
-        <f>C5+C6+C7+C8</f>
-        <v/>
-      </c>
-      <c r="D16" s="12">
-        <f>D5+D6+D7+D8</f>
-        <v/>
-      </c>
-      <c r="F16" s="12">
-        <f>F5+F6+F7+F8</f>
-        <v/>
-      </c>
-      <c r="G16" s="12">
-        <f>G5+G6+G7+G8</f>
-        <v/>
+      <c r="C16" s="12" t="n">
+        <v>83431.14</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <v>84383.17999999999</v>
+      </c>
+      <c r="F16" s="12" t="n">
+        <v>83431.14</v>
+      </c>
+      <c r="G16" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>